<commit_message>
Redesign scoring items for 0.5-point graduated partial credit
Replaces the binary all-or-nothing judgment on 1.0/1.5-point items
with AND-condition or topic-count based rules so every item scores
in 0.5-point steps, matching the requested granularity. 0.5-point
items stay binary since that is already the finest available step.
</commit_message>
<xml_diff>
--- a/scoring_criteria_OBH_Day4.xlsx
+++ b/scoring_criteria_OBH_Day4.xlsx
@@ -436,7 +436,7 @@
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="70" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -477,7 +477,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="300" customHeight="1">
+    <row r="2" ht="320" customHeight="1">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
@@ -497,33 +497,30 @@
       <c r="E2" s="2" t="inlineStr">
         <is>
           <t>環境問題、金融危機・経済環境、P&amp;G等との競争など、ユニリーバを取り巻く外部環境変化に触れているか。
-## 加点条件（いずれか1つ以上に具体的に触れていれば加点）
-- 環境問題（気候変動、資源制約、サステナビリティに対する社会的要請の高まりなど）
-- 金融危機・経済環境（2008年金融危機以降の消費者行動や株主圧力の変化など）
-- P&amp;G等の競合との競争環境（価格競争、コモディティ化、業界内競争の激化など）
-- 上記と同等の、ユニリーバを取り巻く外部環境変化への具体的な言及
-## 0点条件
-- 外部環境の変化に一切触れていない
-- 内部環境（組織文化・体制等）の話のみで外部環境への言及がない
-- 設問と無関係な内容、または回答がない
+## 対象トピック（言及数をカウントする）
+- ① 環境問題（気候変動、資源制約、サステナビリティに対する社会的要請の高まりなど）
+- ② 金融危機・経済環境（2008年金融危機以降の消費者行動や株主圧力の変化など）
+- ③ P&amp;G等の競合との競争環境（価格競争、コモディティ化、業界内競争の激化など）
+- 上記と同等の、ユニリーバを取り巻く外部環境変化への具体的な言及も1トピックとしてカウントする
 ## 判定時の注意
-- 上記トピックすべてを網羅する必要はなく、最低1つの具体的な言及があれば加点する。
-- 「環境問題は重要だ」等、具体性を欠く一般論のみの場合は加点しない。
+- 各トピックは具体的な内容を伴う言及でなければならない。「環境問題は重要だ」等、具体性を欠く一般論のみの言及はカウントしない。
+- 内部環境（組織文化・体制等）の話のみで外部環境への言及がない場合は0.0点とする。
 ## 参考キーワード
 環境問題, 気候変動, サステナビリティ, 金融危機, 2008年, 株主, P&amp;G, 競争, コモディティ化</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>1.0        加点条件のいずれかを満たしている。
-0.0        加点条件をいずれも満たしていない（0点条件に該当）。</t>
+          <t>1.0        トピック①②③のうち2つ以上に具体的に言及している。
+0.5        トピック①②③のうち1つにのみ具体的に言及している。
+0.0        いずれのトピックにも具体的に言及していない（設問と無関係／回答なしを含む）。</t>
         </is>
       </c>
       <c r="G2" s="2" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="3" ht="300" customHeight="1">
+    <row r="3" ht="320" customHeight="1">
       <c r="A3" s="2" t="n">
         <v>1</v>
       </c>
@@ -543,29 +540,26 @@
       <c r="E3" s="2" t="inlineStr">
         <is>
           <t>ターゲット市場の変化により、成功要因が変化していることを指摘しているか。
-## 加点条件
+## 得点条件（両方必須）
 - ターゲット市場の変化（例：先進国中心から新興国・途上国市場への拡大など）に言及している
 - その市場変化に伴い、企業の成功要因（KSF）が変化したこと（例：規模の経済だけでなく持続可能性・社会的信頼が重要になったなど）を明示的に指摘している
-## 0点条件
-- ターゲット市場の変化のみでKSFの変化への言及がない、またはその逆
-- 設問と無関係な内容、または回答がない
 ## 判定時の注意
-- 「KSF」という用語がなくても、実質的に成功要因の変化を説明していれば加点する。
+- 「KSF」という用語がなくても、実質的に成功要因の変化を説明していれば満たすものとする。
 ## 参考キーワード
 新興国, 途上国, ターゲット市場, 成功要因, KSF, 規模の経済, 持続可能性, 社会的信頼</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>0.5        加点条件を満たしている。
-0.0        加点条件を満たしていない（0点条件に該当）。</t>
+          <t>0.5        両方の得点条件を満たしている。
+0.0        どちらか一方のみ、またはいずれにも言及していない（設問と無関係／回答なしを含む）。</t>
         </is>
       </c>
       <c r="G3" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
-    <row r="4" ht="300" customHeight="1">
+    <row r="4" ht="320" customHeight="1">
       <c r="A4" s="2" t="n">
         <v>1</v>
       </c>
@@ -585,16 +579,11 @@
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>USLPをCSRではなく、成長、コスト削減、ブランド向上、供給リスク低減、理念整合などを含む中核戦略として説明しているか。途上国市場の拡大について触れられているか。
-## 加点条件（以下をいずれも満たせば加点）
-- USLPを単なる社会貢献・CSR活動としてではなく、事業成長に資する中核（本業）戦略として説明している
-- 成長、コスト削減、ブランド向上、供給リスク低減、経営理念との整合、のうち少なくとも1つについて具体的な関連を説明している
-- 途上国市場の拡大（新興国での事業機会拡大）についても言及している
-## 0点条件
-- USLPを単なるCSR・社会貢献としてのみ説明している
-- 中核戦略としての位置づけの説明がなく、途上国市場拡大への言及もない
-- 設問と無関係な内容、または回答がない
+## 条件A（0.5点）
+USLPを、成長・コスト削減・ブランド向上・供給リスク低減・経営理念との整合、のうち少なくとも1つと関連付けて、単なるCSR・社会貢献ではなく中核（本業）戦略として説明している。
+## 条件B（0.5点）
+途上国市場の拡大（新興国での事業機会拡大）について言及している。
 ## 判定時の注意
-- 途上国市場拡大への言及が全くない場合は、中核戦略としての論拠が不十分とみなし0点とする。
 - 「CSR」「中核戦略」等の用語ではなく、内容の実質で判断する。
 ## 参考キーワード
 USLP, CSR, 中核戦略, 成長, コスト削減, ブランド, 供給リスク, 理念, 途上国, 新興国市場</t>
@@ -602,15 +591,16 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>1.0        加点条件をすべて満たしている。
-0.0        加点条件を満たしていない（0点条件に該当）。</t>
+          <t>1.0        条件A・Bの両方を満たしている。
+0.5        条件A・Bのいずれか一方のみを満たしている。
+0.0        条件A・Bのいずれも満たしていない（設問と無関係／回答なしを含む）。</t>
         </is>
       </c>
       <c r="G4" s="2" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="5" ht="300" customHeight="1">
+    <row r="5" ht="320" customHeight="1">
       <c r="A5" s="2" t="n">
         <v>1</v>
       </c>
@@ -630,33 +620,27 @@
       <c r="E5" s="2" t="inlineStr">
         <is>
           <t>内向き・保身的な社風、高い地域独立志向、遅い意思決定、既存組織と新戦略の不整合など、自社の組織的課題に触れているか。
-## 加点条件（いずれか1つ以上に具体的に触れていれば加点）
+## 得点条件（いずれか1つ以上）
 - 内向き・保身的な社風
 - 地域組織の独立志向の強さ（地域ごとのサイロ化など）
 - 意思決定の遅さ
 - 既存の組織構造・制度と新戦略（USLP）との不整合
 - 上記と同等の、自社の組織的課題への具体的な言及
-## 0点条件
-- 組織的課題への言及が一切ない
-- 外部環境の話のみで内部組織課題への言及がない
-- 設問と無関係な内容、または回答がない
-## 判定時の注意
-- 例示された課題のうち、最低1つに具体的な言及があれば加点する。
 ## 参考キーワード
 内向き, 保身的, 社風, 地域独立志向, サイロ化, 意思決定の遅さ, 組織構造, 新戦略との不整合</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>0.5        加点条件のいずれかを満たしている。
-0.0        加点条件をいずれも満たしていない（0点条件に該当）。</t>
+          <t>0.5        得点条件のいずれかを満たしている。
+0.0        いずれの条件も満たしていない（外部環境のみの言及、設問と無関係、回答なしを含む）。</t>
         </is>
       </c>
       <c r="G5" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
-    <row r="6" ht="300" customHeight="1">
+    <row r="6" ht="320" customHeight="1">
       <c r="A6" s="2" t="n">
         <v>2</v>
       </c>
@@ -676,31 +660,31 @@
       <c r="E6" s="2" t="inlineStr">
         <is>
           <t>コッターの8ステップ、またはレヴィンのモデル等を使い、変革の進め方を分析しているか。
-## 加点条件
-- コッターの8ステップモデル、レヴィンの変革モデル（解凍・変革・再凍結）、またはこれらに準ずる変革プロセスのフレームワークを用いている
-- フレームワークの段階（一部でも可）に沿って、USLPの変革の進め方を具体的に分析している（フレームワーク名の列挙のみは不可）
-## 0点条件
-- フレームワークへの言及がなく、段階的な変革プロセスの分析もされていない
-- フレームワーク名のみを挙げて、ケースの内容と紐づいた分析がない
-- 設問と無関係な内容、または回答がない
+## 条件A（0.5点）
+コッターの8ステップモデル、レヴィンの変革モデル（解凍・変革・再凍結）、またはこれらに準ずる変革プロセスのフレームワークを提示している。
+## 条件B（0.5点）
+フレームワークの複数の段階に沿って、USLPの変革の進め方を具体的に分析している（フレームワーク名の列挙のみでは満たさない）。
+## 条件C（0.5点）
+分析がケース内の具体的な出来事・取り組み（例：ULEの新設、ブランド・インプリント、CB4Lワークショップ、USLPリフレッシュ等）と結び付けられている。
 ## 判定時の注意
-- フレームワーク名を明示していなくても、実質的に同等の段階的分析がなされていれば加点してよい。
-- フレームワークの一部の段階のみの分析であっても、具体的な分析があれば加点する。
+- フレームワーク名を明示していなくても、実質的に同等の段階的分析がなされていれば条件Aを満たすものとする。
 ## 参考キーワード
 コッター, 8ステップ, レヴィン, 解凍, 変革, 再凍結, 変革プロセス</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>1.5        加点条件を満たしている。
-0.0        加点条件を満たしていない（0点条件に該当）。</t>
+          <t>1.5        条件A・B・Cをすべて満たしている。
+1.0        条件のうち2つを満たしている。
+0.5        条件のうち1つを満たしている。
+0.0        いずれの条件も満たしていない（設問と無関係／回答なしを含む）。</t>
         </is>
       </c>
       <c r="G6" s="2" t="n">
         <v>1.5</v>
       </c>
     </row>
-    <row r="7" ht="300" customHeight="1">
+    <row r="7" ht="320" customHeight="1">
       <c r="A7" s="2" t="n">
         <v>2</v>
       </c>
@@ -720,30 +704,28 @@
       <c r="E7" s="2" t="inlineStr">
         <is>
           <t>7S等で、USLP戦略と組織構造・制度・人材・スキル・価値観・スタイルなどの整合／不整合を分析しているか。
-## 加点条件
-- 7Sフレームワーク（Strategy / Structure / Systems / Staff / Skills / Style / Shared Value等）、またはこれに準ずる枠組みを用いている
-- 組織構造・制度・人材・スキル・価値観・スタイルのうち、少なくとも1つの要素について、USLP戦略との整合または不整合を具体的に分析している
-## 0点条件
-- フレームワークへの言及・要素別の分析がともにない
-- フレームワーク名のみで、具体的な整合／不整合の分析がない
-- 設問と無関係な内容、または回答がない
+## 条件A（0.5点）
+7Sフレームワーク（Strategy / Structure / Systems / Staff / Skills / Style / Shared Value等）、またはこれに準ずる枠組みを提示している。
+## 条件B（0.5点）
+組織構造・制度・人材・スキル・価値観・スタイルのうち、少なくとも1つの要素について、USLP戦略との整合または不整合を具体的に分析している。
 ## 判定時の注意
-- 「7S」という用語がなくても、複数の組織要素（構造・人材・価値観等）とUSLP戦略との整合性を分析していれば加点してよい。
+- 「7S」という用語がなくても、複数の組織要素（構造・人材・価値観等）とUSLP戦略との整合性を分析していれば条件Aを満たすものとする。
 ## 参考キーワード
 7S, Strategy, Structure, Systems, Staff, Skills, Style, Shared Value, 組織整合</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>1.0        加点条件を満たしている。
-0.0        加点条件を満たしていない（0点条件に該当）。</t>
+          <t>1.0        条件A・Bの両方を満たしている。
+0.5        条件A・Bのいずれか一方のみを満たしている。
+0.0        条件A・Bのいずれも満たしていない（設問と無関係／回答なしを含む）。</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="8" ht="300" customHeight="1">
+    <row r="8" ht="320" customHeight="1">
       <c r="A8" s="2" t="n">
         <v>2</v>
       </c>
@@ -763,32 +745,30 @@
       <c r="E8" s="2" t="inlineStr">
         <is>
           <t>ポールマンのリーダーシップスタイル、パスゴール理論当てはめ、リーダー行動の変化、変革コミュニケーションに触れているか。
-## 加点条件（以下のうち少なくとも1つに具体的に触れていれば加点）
-- ポールマンのリーダーシップスタイルの特徴づけ（例：変革型リーダーシップ、長期志向、理念重視など）
-- パスゴール理論（指示型・支援型・参加型・達成志向型等）へのあてはめ
-- 変革過程におけるリーダー行動の変化（例：初期のトップダウン的関与から徐々に権限委譲するなど）
-- 変革を推進するためのコミュニケーション（ビジョンの発信、社内外への説明など）
-## 0点条件
-- リーダーシップに関する言及が一切ない
-- 単なる感想（例：「素晴らしいリーダーだと思う」）のみで、分析的な言及がない
-- 設問と無関係な内容、または回答がない
+## 対象トピック（言及数をカウントする）
+- ① ポールマンのリーダーシップスタイルの特徴づけ（例：変革型リーダーシップ、長期志向、理念重視など）
+- ② パスゴール理論（指示型・支援型・参加型・達成志向型等）へのあてはめ
+- ③ 変革過程におけるリーダー行動の変化（例：初期のトップダウン的関与から徐々に権限委譲するなど）
+- ④ 変革を推進するためのコミュニケーション（ビジョンの発信、社内外への説明など）
 ## 判定時の注意
-- 上記4トピックのうち最低1つについて具体的な分析があれば加点する。
+- 単なる感想（例：「素晴らしいリーダーだと思う」）のみで分析的な言及がない場合はカウントしない。
 ## 参考キーワード
 ポールマン, リーダーシップスタイル, パスゴール理論, リーダー行動, 権限委譲, 変革コミュニケーション</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>1.5        加点条件を満たしている。
-0.0        加点条件を満たしていない（0点条件に該当）。</t>
+          <t>1.5        トピック①〜④のうち3つ以上に具体的に言及している。
+1.0        トピック①〜④のうち2つに具体的に言及している。
+0.5        トピック①〜④のうち1つにのみ具体的に言及している。
+0.0        いずれにも言及していない（設問と無関係／回答なしを含む）。</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">
         <v>1.5</v>
       </c>
     </row>
-    <row r="9" ht="300" customHeight="1">
+    <row r="9" ht="320" customHeight="1">
       <c r="A9" s="2" t="n">
         <v>3</v>
       </c>
@@ -808,17 +788,12 @@
       <c r="E9" s="2" t="inlineStr">
         <is>
           <t>2015年時点の選択肢として、C「社外パートナーシップの構築に集中する」を明確に選択しているか。
-## 加点条件
+## 得点条件（いずれかに該当）
 - 「C」を選択していることが明確に書かれている
 - 「社外パートナーシップの構築に集中する」と同等の内容を選んでいる
 - 「変革の方向を転換し、外部との連携を強める」といった、選択肢Cに相当する内容を選んでいる
-## 0点条件
-- AまたはBを選択している
-- 複数案を併記しており、最終的な選択が不明確
-- 「状況による」「どれでもない」など、選択が明確でない
-- 設問3への回答がない
 ## 判定時の注意
-- 「C」という記号がなくても、内容が選択肢Cに相当すれば加点してよい。
+- 「C」という記号がなくても、内容が選択肢Cに相当すれば満点としてよい。
 - 一方で、Cに近い言葉が一部あっても、最終判断がAまたはBであれば0点とする。
 ## 参考キーワード
 C, 外部パートナーシップ, 社外連携, 変革の方向転換</t>
@@ -826,15 +801,15 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>0.5        加点条件を満たしている。
-0.0        加点条件を満たしていない（0点条件に該当）。</t>
+          <t>0.5        得点条件のいずれかを満たしている。
+0.0        AまたはBを選択、選択が不明確、または設問3への回答がない。</t>
         </is>
       </c>
       <c r="G9" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
-    <row r="10" ht="300" customHeight="1">
+    <row r="10" ht="320" customHeight="1">
       <c r="A10" s="2" t="n">
         <v>3</v>
       </c>
@@ -854,18 +829,13 @@
       <c r="E10" s="2" t="inlineStr">
         <is>
           <t>選択肢の比較や分析結果を踏まえて、意思決定の根拠を説明しているか。
-## 加点条件（以下のうち1つ以上に該当する理由が述べられていれば加点）
+## 得点条件（いずれか1つ以上）
 - A案は、取り組みを2倍に強化するため、短期業績の悪化や投資負担が大きいと説明している
 - B案は、USLPの理念・哲学・ビジョンと矛盾し、社員やステークホルダーの不信を招くと説明している
 - GHG排出量や水使用量などの課題は、ユニリーバ単独では達成が難しいと説明している
 - バリューチェーン前後の協力、消費者行動の変容、NGO・政府・業界団体などとの連携が必要だと説明している
 - C案は、USLPの理念を維持しながら、実行方法を現実的に転換する選択だと説明している
 - 外部パートナーシップにより、環境・社会課題への影響力を広げられると説明している
-## 0点条件
-- 理由が書かれていない
-- 「Cがよいと思うから」など、根拠が実質的にない
-- 設問と無関係な理由である
-- 事実や分析に基づく説明がなく、感想にとどまっている
 ## 判定時の注意
 - この項目は、選択肢Cを選んでいるかとは独立して採点する。
 - AまたはBを選んでいても、選択肢比較や分析に基づく理由が述べられていれば0.5点を与えてよい。
@@ -876,15 +846,15 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>0.5        加点条件のいずれかを満たしている（設問3-1の選択結果とは独立に判定）。
-0.0        加点条件をいずれも満たしていない（0点条件に該当）。</t>
+          <t>0.5        得点条件のいずれかを満たしている（設問3-1の選択結果とは独立に判定）。
+0.0        理由が書かれていない、根拠が実質的にない、または設問と無関係。</t>
         </is>
       </c>
       <c r="G10" s="2" t="n">
         <v>0.5</v>
       </c>
     </row>
-    <row r="11" ht="300" customHeight="1">
+    <row r="11" ht="320" customHeight="1">
       <c r="A11" s="2" t="n">
         <v>4</v>
       </c>
@@ -904,26 +874,23 @@
       <c r="E11" s="2" t="inlineStr">
         <is>
           <t>設問3で選んだオプションを実行するための具体的なアクションが述べられているか。
-## 加点条件（以下の要素のうち2要素以上が回答に含まれていれば加点）
-- 行動（何をするかが具体的に書かれている）：例）提携する、協議体を作る、共同プロジェクトを立ち上げる、KPIを設定する、啓発キャンペーンを行う、サプライヤー基準を見直す、進捗を開示する、社員に説明するなど
-- 方法・順序・運用（どのように進めるかが書かれている）：例）短期・中期で段階的に進める、優先領域を決める、定期的にモニタリングする、成果を公表する、パイロットを行ってから展開する、責任者を置くなど
-## 0点条件
-- 「頑張る」「リーダーシップを発揮する」「社員を巻き込む」など、抽象的な方針だけで具体的な行動がない
-- アクションではなく、設問3の理由説明にとどまっている
-- 誰に何をするのかがほとんど読み取れない
-- 設問と無関係な内容である
-- 回答がない、またはテキストが50文字以下
+## 条件A（0.5点）：行動
+何をするかが具体的に書かれている。例）提携する、協議体を作る、共同プロジェクトを立ち上げる、KPIを設定する、啓発キャンペーンを行う、サプライヤー基準を見直す、進捗を開示する、社員に説明するなど
+## 条件B（0.5点）：方法・順序・運用
+どのように進めるかが書かれている。例）短期・中期で段階的に進める、優先領域を決める、定期的にモニタリングする、成果を公表する、パイロットを行ってから展開する、責任者を置くなど
 ## 判定時の注意
-- 短い回答でも、行動・方法のうち2要素以上が明確であれば1.0点を与える。
-- 長い回答でも、抽象論や感想にとどまり、具体的な実行内容がなければ0点とする。
+- 「頑張る」「リーダーシップを発揮する」「社員を巻き込む」など抽象的な方針だけで具体的な行動がない場合は満たさない。
+- アクションではなく設問3の理由説明にとどまっている場合は満たさない。
+- 回答がない、またはテキストが50文字以下の場合は0.0点とする。
 ## 参考キーワード
 提携, 協議体, 共同プロジェクト, KPI, 啓発キャンペーン, サプライヤー基準, モニタリング, パイロット, 責任者</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>1.0        加点条件（2要素以上）を満たしている。
-0.0        加点条件を満たしていない（0点条件に該当）。</t>
+          <t>1.0        条件A・Bの両方を満たしている。
+0.5        条件A・Bのいずれか一方のみを満たしている。
+0.0        条件A・Bのいずれも満たしていない（50文字以下・設問と無関係・回答なしを含む）。</t>
         </is>
       </c>
       <c r="G11" s="2" t="n">

</xml_diff>

<commit_message>
Add score-band feedback messages for each question group
Mirrors the CRT workbook's "フィードバック文言案ver2" tab: for each
of the 4 question groups, provides tiered feedback text keyed to the
group's point total, as a markdown bank and a matching xlsx sheet.
Wires the feedback bank into the main grading prompt's output format.
</commit_message>
<xml_diff>
--- a/scoring_criteria_OBH_Day4.xlsx
+++ b/scoring_criteria_OBH_Day4.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="採点基準_OBH_Day4" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="フィードバック文言案" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,7 +30,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -40,6 +41,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
         <bgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -55,12 +62,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -900,4 +910,232 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>フィードバック分類</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>満点</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>フィードバック文言</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>設問1：外部・内部環境分析</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>2.5点以上であれば</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>1.0点以上2.5点未満であれば</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>1.0点未満であれば</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="260" customHeight="1">
+      <c r="A3" s="2" t="n"/>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>ポールマンがUSLP戦略を打ち出した背景を、外部環境（サステナビリティへの社会的要請、金融危機後の株主行動の変化、P&amp;Gなど競合との競争激化）と内部環境（内向きな社風、地域組織の独立志向、意思決定の遅さなど）の両面から、多角的かつ具体的に説明できています。また、USLPを単なるCSRではなく成長・コスト削減・ブランド価値向上などに資する中核戦略として位置づけ、途上国市場の拡大という機会にも言及できており、なぜ「今」この戦略が必要だったのかという説得力のある論理構成になっています。
+実務においても、大きな戦略転換を提案する際は、今回のように外部環境（市場・競合・社会的要請）と内部環境（組織文化・意思決定プロセス）の両方を押さえたうえで、その戦略が「本業の成長」にどう資するのかを語れると、周囲の納得感を得やすくなります。ぜひこの視点を今後の実務でも意識してみてください。</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>USLP戦略の背景について、外部環境・内部環境のいずれか一方、あるいはUSLPの戦略的位置づけについて部分的に説明できていますが、まだ論点の一部にとどまっています。例えば、外部環境（社会的要請、金融危機、競合動向）と内部環境（社風、意思決定の遅さ、組織の独立志向）の両方に触れる、あるいはUSLPを成長・コスト削減などの具体的な経営指標と結び付けて中核戦略として説明する、といった点を補強すると、より説得力のある分析になります。
+戦略転換の必然性を語る際は、「なぜ外部から見て必要か」「なぜ社内から見て必要か」の両輪で考える習慣をつけると、片方だけの説明で終わらず、相手にとってより納得感のある提案ができるようになります。</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>USLP戦略の背景説明について、外部環境・内部環境への具体的な言及、およびUSLPを中核戦略として位置づける説明が、まだ十分ではありません。ケースの記述に立ち返り、①ユニリーバを取り巻く外部環境（社会の要請、金融危機後の株主行動、P&amp;Gなど競合の動き）、②社内の組織的課題（内向きな社風、地域組織の独立志向、意思決定の遅さ）、③USLPが単なる社会貢献ではなく成長・コスト削減等に資する中核戦略であること、④途上国市場拡大という機会、の4点を意識して整理し直してみてください。
+戦略の背景を分析する際は、外部環境分析（PEST、5フォース等）と内部環境分析（組織文化、意思決定プロセス等）を型として身につけておくと、初見のケースでも論点の抜け漏れを防ぎやすくなります。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>設問2：変革プロセス・組織・リーダーシップ分析</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>3.0点以上であれば</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>1.5点以上3.0点未満であれば</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>1.5点未満であれば</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="260" customHeight="1">
+      <c r="A5" s="2" t="n"/>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>USLP実行の4年間を評価するにあたり、コッターの8ステップやレヴィンのモデルなどの変革フレームワークを使って変革プロセスを具体的に分析し、7S等を用いて組織構造・人材・価値観とUSLP戦略との整合／不整合まで踏み込んで検討できています。さらに、ポールマンのリーダーシップスタイルやリーダー行動の変化、変革コミュニケーションについても具体的に言及できており、変革を「プロセス」「組織」「リーダーシップ」の複数の視点から多面的に評価する、質の高い分析になっています。
+実務で変革を推進する立場に立った際も、フレームワークを型として使いながら、組織の各要素（構造・人材・価値観）の整合性やリーダー自身の行動・発信のあり方まで含めて振り返る習慣は、変革の成否を見極めるうえで非常に有効です。</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>変革プロセスや組織整合、リーダーシップのいずれかについては具体的な分析ができていますが、他の観点についてはフレームワークの名称にとどまっていたり、ケースの具体的な出来事と結び付いていなかったりする部分が見られます。例えば、コッターやレヴィンのモデルを使う場合は、単に名称を挙げるだけでなく、ULEの新設やCB4Lワークショップなど、ケース内の具体的な取り組みをどの段階に位置づけられるかまで踏み込むと、分析に厚みが出ます。また、7S分析やパスゴール理論についても、具体的な組織要素やリーダー行動と結び付けて説明できると、評価がより説得力を持ちます。
+複数のフレームワークを「知っている」ことと「ケースの事実に当てはめて使いこなす」ことの間には差があります。この差を埋める意識を持って、今後も分析の練習を重ねてみてください。</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>変革プロセス、組織整合、リーダーシップのいずれについても、具体的な分析がまだ十分ではありません。まずはコッターの8ステップやレヴィンのモデルを使って、USLP実行の4年間がどのように進んだのかを段階的に整理し、次に7S等の枠組みで組織構造・人材・価値観とUSLP戦略の整合性を確認し、最後にポールマンのリーダーシップスタイルや行動の変化、コミュニケーションのあり方を振り返る、という3つのステップで分析を組み立て直してみてください。
+フレームワークは、複雑な変革プロセスを整理し、見落としを防ぐための強力な道具です。まずは型に沿って考える練習を重ね、その後にケースの具体的な事実と結び付ける訓練をしていくとよいでしょう。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>設問3：意思決定</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>1.0点であれば</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>0.5点であれば</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>0.0点であれば</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="260" customHeight="1">
+      <c r="A7" s="2" t="n"/>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>2015年時点の選択肢として、外部パートナーシップの構築に集中する「C」を明確に選択し、その理由についても、A案・B案それぞれのリスクや、ユニリーバ単独では目標達成が難しいという構造的な課題、外部との連携による影響力拡大の可能性など、複数の観点から比較検討したうえで説明できています。単なる好みではなく、選択肢の比較と分析に基づいた意思決定ができている点が評価できます。
+実務における意思決定でも、複数の選択肢のメリット・デメリットを比較したうえで、なぜその選択が他よりも優れているのかを論理的に説明する姿勢は、周囲の納得感を得るうえで非常に重要です。</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>選択肢の選択、またはその理由説明のいずれか一方については基準を満たしていますが、両方を満たすには至っていません。例えば、Cを選んだものの理由が「なんとなく良さそうだから」にとどまっている場合や、逆に説得力のある理由を述べているものの最終的な選択が不明確な場合が該当します。意思決定においては、「何を選ぶか」と「なぜそれを選ぶか」の両方が揃って初めて、説得力のある提案になります。
+A・B・Cそれぞれの選択肢を選んだ場合に何が起こりうるかを比較したうえで、最終的な結論を明確に述べる、という流れを意識してみてください。</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>2015年時点の意思決定について、選択肢の選択、およびその理由説明のいずれも、まだ基準を満たしていません。まずはA・B・Cそれぞれの選択肢を選んだ場合に何が起こりうるかを比較し、そのうえでどれか一つを明確に選び、その根拠を説明する、という基本的な意思決定の流れを踏んでみてください。
+複数の選択肢を比較検討せずに結論を出してしまうと、なぜその選択が最善なのかを他者に説明することが難しくなります。今後の意思決定の場面でも、複数の選択肢を比較する習慣を意識してみてください。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>設問4：アクションプラン</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>1.0点であれば</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>0.5点であれば</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>0.0点であれば</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="260" customHeight="1">
+      <c r="A9" s="2" t="n"/>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>選択したオプションを実行するための具体的なアクションについて、「何をするか」という行動と、「どのように進めるか」という方法・順序の両方を具体的に述べることができています。抽象的な方針にとどまらず、実行可能なレベルまで具体化できている点が評価できます。
+実務においても、アクションプランを立てる際は「誰が」「何を」「どのように」「いつまでに」を明確にすることで、計画が絵に描いた餅にならず、実行に移しやすくなります。今回のような具体性を今後も意識してみてください。</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>「何をするか」という具体的な行動、または「どのように進めるか」という方法・順序のいずれか一方については具体的に述べられていますが、両方を満たすには至っていません。例えば、提携や協議体の設立など具体的な行動は挙げられているものの、それをどのような順序や体制で進めるかが書かれていない場合や、逆に進め方は書かれているものの、具体的に何を行うのかが曖昧な場合が該当します。
+アクションプランを書く際は、「行動」と「進め方」の両方をセットで考える習慣をつけると、計画の実行可能性がぐっと高まります。</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>「頑張る」「リーダーシップを発揮する」といった抽象的な方針にとどまっており、具体的な行動や進め方がまだ読み取れません。誰に対して、何を、どのように行うのかを、具体的な単語（提携する、協議体を作る、KPIを設定する、段階的に展開する等）を使って書き直してみてください。
+抽象的な方針だけでは、実際に何をすればよいのかが読み手に伝わりません。実行可能なレベルまで具体化する練習を重ねてみてください。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Expand xlsx feedback sheet to cover all score bands
Previously only the top score-band feedback was mirrored into the
xlsx per question group; the middle and bottom bands existed only in
feedback_messages.md. Adds all 3 tiers per question (12 tiers total)
so the xlsx is a complete standalone reference matching the md file.
</commit_message>
<xml_diff>
--- a/scoring_criteria_OBH_Day4.xlsx
+++ b/scoring_criteria_OBH_Day4.xlsx
@@ -931,7 +931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1010,15 +1010,15 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>設問2：変革プロセス・組織・リーダーシップ分析</t>
+          <t>設問1：外部・内部環境分析</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>3.0点以上であれば</t>
+          <t>1.0点以上2.5点未満であれば</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -1037,8 +1037,8 @@
       <c r="B5" s="2" t="n"/>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>USLP実行の4年間を評価するにあたり、コッターの8ステップやレヴィンのモデルなどの変革フレームワークを使って変革プロセスを具体的に分析し、7S等を用いて組織構造・人材・価値観とUSLP戦略との整合／不整合まで踏み込んで検討できています（USLP実施前後で各組織要素を対比しながら変化を具体的に示せている点も評価できます）。さらに、ポールマンのリーダーシップスタイルやリーダー行動の変化、変革コミュニケーションについても具体的に言及できており、変革を「プロセス」「組織」「リーダーシップ」の複数の視点から多面的に評価する、質の高い分析になっています。
-実務で変革を推進する立場に立った際も、フレームワークを型として使いながら、組織の各要素（構造・人材・価値観）の整合性やリーダー自身の行動・発信のあり方まで含めて振り返る習慣は、変革の成否を見極めるうえで非常に有効です。</t>
+          <t>USLP戦略の背景について、外部環境・内部環境のいずれか一方、あるいはUSLPの戦略的位置づけについて部分的に説明できていますが、まだ論点の一部にとどまっています。例えば、外部環境（社会的要請、金融危機、競合動向）と内部環境（社風、意思決定の遅さ、組織の独立志向）の両方に触れる、あるいはUSLPを成長・コスト削減などの具体的な経営指標と結び付けて中核戦略として説明する、といった点を補強すると、より説得力のある分析になります。
+戦略転換の必然性を語る際は、「なぜ外部から見て必要か」「なぜ社内から見て必要か」の両輪で考える習慣をつけると、片方だけの説明で終わらず、相手にとってより納得感のある提案ができるようになります。</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1057,15 +1057,15 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>設問3：意思決定</t>
+          <t>設問1：外部・内部環境分析</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>1.0点であれば</t>
+          <t>1.0点未満であれば</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -1084,8 +1084,8 @@
       <c r="B7" s="2" t="n"/>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>2015年時点の選択肢として、外部パートナーシップの構築に集中する「C」を明確に選択し、その理由についても、A案・B案それぞれのリスクや、ユニリーバ単独では目標達成が難しいという構造的な課題、外部との連携による影響力拡大の可能性など、複数の観点から比較検討したうえで説明できています。単なる好みではなく、選択肢の比較と分析に基づいた意思決定ができている点が評価できます。
-実務における意思決定でも、複数の選択肢のメリット・デメリットを比較したうえで、なぜその選択が他よりも優れているのかを論理的に説明する姿勢は、周囲の納得感を得るうえで非常に重要です。</t>
+          <t>USLP戦略の背景説明について、外部環境・内部環境への具体的な言及、およびUSLPを中核戦略として位置づける説明が、まだ十分ではありません。ケースの記述に立ち返り、①ユニリーバを取り巻く外部環境（社会の要請、金融危機後の株主行動、P&amp;Gなど競合の動き）、②社内の組織的課題（内向きな社風、地域組織の独立志向、意思決定の遅さ）、③USLPが単なる社会貢献ではなく成長・コスト削減等に資する中核戦略であること、④途上国市場拡大という機会、の4点を意識して整理し直してみてください。
+戦略の背景を分析する際は、外部環境分析（PEST、5フォース等）と内部環境分析（組織文化、意思決定プロセス等）を型として身につけておくと、初見のケースでも論点の抜け漏れを防ぎやすくなります。</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1104,15 +1104,15 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>設問4：アクションプラン</t>
+          <t>設問2：変革プロセス・組織・リーダーシップ分析</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>1.0点であれば</t>
+          <t>3.0点以上であれば</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -1131,17 +1131,201 @@
       <c r="B9" s="2" t="n"/>
       <c r="C9" s="2" t="inlineStr">
         <is>
+          <t>USLP実行の4年間を評価するにあたり、コッターの8ステップやレヴィンのモデルなどの変革フレームワークを使って変革プロセスを具体的に分析し、7S等を用いて組織構造・人材・価値観とUSLP戦略との整合／不整合まで踏み込んで検討できています（USLP実施前後で各組織要素を対比しながら変化を具体的に示せている点も評価できます）。さらに、ポールマンのリーダーシップスタイルやリーダー行動の変化、変革コミュニケーションについても具体的に言及できており、変革を「プロセス」「組織」「リーダーシップ」の複数の視点から多面的に評価する、質の高い分析になっています。
+実務で変革を推進する立場に立った際も、フレームワークを型として使いながら、組織の各要素（構造・人材・価値観）の整合性やリーダー自身の行動・発信のあり方まで含めて振り返る習慣は、変革の成否を見極めるうえで非常に有効です。</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>「何をするか」という具体的な行動、または「どのように進めるか」という方法・順序のいずれか一方については具体的に述べられていますが、両方を満たすには至っていません。例えば、提携や協議体の設立など具体的な行動は挙げられているものの、それをどのような順序や体制で進めるかが書かれていない場合や、逆に進め方は書かれているものの、具体的に何を行うのかが曖昧な場合が該当します。
+アクションプランを書く際は、「行動」と「進め方」の両方をセットで考える習慣をつけると、計画の実行可能性がぐっと高まります。</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>「頑張る」「リーダーシップを発揮する」といった抽象的な方針にとどまっており、具体的な行動や進め方がまだ読み取れません。誰に対して、何を、どのように行うのかを、具体的な単語（提携する、協議体を作る、KPIを設定する、段階的に展開する等）を使って書き直してみてください。
+抽象的な方針だけでは、実際に何をすればよいのかが読み手に伝わりません。実行可能なレベルまで具体化する練習を重ねてみてください。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>設問2：変革プロセス・組織・リーダーシップ分析</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1.5点以上3.0点未満であれば</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>変革プロセスや組織整合、リーダーシップのいずれかについては具体的な分析ができていますが、他の観点についてはフレームワークの名称にとどまっていたり、ケースの具体的な出来事と結び付いていなかったりする部分が見られます。例えば、コッターやレヴィンのモデルを使う場合は、単に名称を挙げるだけでなく、ULEの新設やCB4Lワークショップなど、ケース内の具体的な取り組みをどの段階に位置づけられるかまで踏み込むと、分析に厚みが出ます。また、7S分析についても、「一貫性がある」「整合している」といった結論だけで終わらせず、USLP実施前後で組織構造・人材・価値観などの各要素がどう変化したかを個別に対比して示すと、評価がより説得力を持ちます。パスゴール理論についても、具体的なリーダー行動と結び付けて説明できるとよいでしょう。
+複数のフレームワークを「知っている」ことと「ケースの事実に当てはめて使いこなす」ことの間には差があります。この差を埋める意識を持って、今後も分析の練習を重ねてみてください。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>設問2：変革プロセス・組織・リーダーシップ分析</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1.5点未満であれば</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>変革プロセス、組織整合、リーダーシップのいずれについても、具体的な分析がまだ十分ではありません。まずはコッターの8ステップやレヴィンのモデルを使って、USLP実行の4年間がどのように進んだのかを段階的に整理し、次に7S等の枠組みで組織構造・人材・価値観とUSLP戦略の整合性を確認し、最後にポールマンのリーダーシップスタイルや行動の変化、コミュニケーションのあり方を振り返る、という3つのステップで分析を組み立て直してみてください。
+フレームワークは、複雑な変革プロセスを整理し、見落としを防ぐための強力な道具です。まずは型に沿って考える練習を重ね、その後にケースの具体的な事実と結び付ける訓練をしていくとよいでしょう。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>設問3：意思決定</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1.0点であれば</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2015年時点の選択肢として、外部パートナーシップの構築に集中する「C」を明確に選択し、その理由についても、A案・B案それぞれのリスクや、ユニリーバ単独では目標達成が難しいという構造的な課題、外部との連携による影響力拡大の可能性など、複数の観点から比較検討したうえで説明できています。単なる好みではなく、選択肢の比較と分析に基づいた意思決定ができている点が評価できます。
+実務における意思決定でも、複数の選択肢のメリット・デメリットを比較したうえで、なぜその選択が他よりも優れているのかを論理的に説明する姿勢は、周囲の納得感を得るうえで非常に重要です。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>設問3：意思決定</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>0.5点であれば</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>選択肢の選択、またはその理由説明のいずれか一方については基準を満たしていますが、両方を満たすには至っていません。例えば、Cを選んだものの理由が「なんとなく良さそうだから」にとどまっている場合や、逆に説得力のある理由を述べているものの最終的な選択が不明確な場合が該当します。意思決定においては、「何を選ぶか」と「なぜそれを選ぶか」の両方が揃って初めて、説得力のある提案になります。
+A・B・Cそれぞれの選択肢を選んだ場合に何が起こりうるかを比較したうえで、最終的な結論を明確に述べる、という流れを意識してみてください。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>設問3：意思決定</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>0.0点であれば</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2015年時点の意思決定について、選択肢の選択、およびその理由説明のいずれも、まだ基準を満たしていません。まずはA・B・Cそれぞれの選択肢を選んだ場合に何が起こりうるかを比較し、そのうえでどれか一つを明確に選び、その根拠を説明する、という基本的な意思決定の流れを踏んでみてください。
+複数の選択肢を比較検討せずに結論を出してしまうと、なぜその選択が最善なのかを他者に説明することが難しくなります。今後の意思決定の場面でも、複数の選択肢を比較する習慣を意識してみてください。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>設問4：アクションプラン</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1.0点であれば</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="C21" t="inlineStr">
+        <is>
           <t>選択したオプションを実行するための具体的なアクションについて、「何をするか」という行動と、「どのように進めるか」という方法・順序の両方を具体的に述べることができています。抽象的な方針にとどまらず、実行可能なレベルまで具体化できている点が評価できます。
 実務においても、アクションプランを立てる際は「誰が」「何を」「どのように」「いつまでに」を明確にすることで、計画が絵に描いた餅にならず、実行に移しやすくなります。今回のような具体性を今後も意識してみてください。</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>設問4：アクションプラン</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>0.5点であれば</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="C23" t="inlineStr">
         <is>
           <t>「何をするか」という具体的な行動、または「どのように進めるか」という方法・順序のいずれか一方については具体的に述べられていますが、両方を満たすには至っていません。例えば、提携や協議体の設立など具体的な行動は挙げられているものの、それをどのような順序や体制で進めるかが書かれていない場合や、逆に進め方は書かれているものの、具体的に何を行うのかが曖昧な場合が該当します。
 アクションプランを書く際は、「行動」と「進め方」の両方をセットで考える習慣をつけると、計画の実行可能性がぐっと高まります。</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>設問4：アクションプラン</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>0.0点であれば</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="C25" t="inlineStr">
         <is>
           <t>「頑張る」「リーダーシップを発揮する」といった抽象的な方針にとどまっており、具体的な行動や進め方がまだ読み取れません。誰に対して、何を、どのように行うのかを、具体的な単語（提携する、協議体を作る、KPIを設定する、段階的に展開する等）を使って書き直してみてください。
 抽象的な方針だけでは、実際に何をすればよいのかが読み手に伝わりません。実行可能なレベルまで具体化する練習を重ねてみてください。</t>

</xml_diff>